<commit_message>
hmm yeah lowkey have forgotten what ive changed i think ive not really actually changed anything but just accidental reruns etc ive editted the way in comp 1 that the supersets are made b10brf and b10brm have been combined for same strain same epitope so we have 15 comparisons now rather than 2 sets of 6
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Superset/Kb_pc_values_CDR3.xlsx
+++ b/Final_Figures_and_Sheets_Superset/Kb_pc_values_CDR3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>B10BRF|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>B10BRF|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1647,15 +1647,15 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.008157169117647059</v>
+        <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>B10BRF|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>(2,3)</t>
+          <t>(1,4)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -1689,15 +1689,15 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.004111842105263158</v>
+        <v>0.0003734129947722181</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>B10BRM|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>(4,5)</t>
+          <t>(1,5)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -1731,15 +1731,15 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.003534145280556764</v>
+        <v>8.023750300890636e-05</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>B10BRM|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>(4,6)</t>
+          <t>(1,6)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -1773,15 +1773,15 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.010092180546726</v>
+        <v>0.008157169117647059</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>B10BRM|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>(5,6)</t>
+          <t>(2,3)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -1815,15 +1815,15 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.001382998340401992</v>
+        <v>0.0005653782894736842</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BALBc|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>(7,8)</t>
+          <t>(2,4)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -1857,15 +1857,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.002615933412604043</v>
+        <v>0.0003004807692307692</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>BALBc|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>(7,9)</t>
+          <t>(2,5)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -1899,15 +1899,15 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.006896551724137931</v>
+        <v>0.03254132231404959</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BALBc|RTY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>(8,9)</t>
+          <t>(2,6)</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -1936,30 +1936,30 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.00558477823235275</v>
+        <v>4.837461300309598e-05</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>B10BRF|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>(10,11)</t>
+          <t>(3,4)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -1978,30 +1978,30 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.01888810884899542</v>
+        <v>0.0005656108597285068</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>B10BRF|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>(10,12)</t>
+          <t>(3,5)</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2020,30 +2020,30 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.008229613004148813</v>
+        <v>0.001276130286825474</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B10BRF|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>(11,12)</t>
+          <t>(3,6)</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -2062,30 +2062,30 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.001865418532085199</v>
+        <v>0.004111842105263158</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>B10BRM|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>(13,14)</t>
+          <t>(4,5)</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2104,30 +2104,30 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.005793526201689467</v>
+        <v>0.003534145280556764</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>B10BRM|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>(13,15)</t>
+          <t>(4,6)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2146,30 +2146,30 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.001847652641303435</v>
+        <v>0.010092180546726</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>B10BRM|SNY</t>
+          <t>B10BR|RTY</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>(14,15)</t>
+          <t>(5,6)</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -2188,7 +2188,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2197,21 +2197,21 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.005734666759913281</v>
+        <v>0.001382998340401992</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>BALBc|SNY</t>
+          <t>BALBc|RTY</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>(16,17)</t>
+          <t>(7,8)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2230,7 +2230,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2239,21 +2239,21 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.005484237894052649</v>
+        <v>0.002615933412604043</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>BALBc|SNY</t>
+          <t>BALBc|RTY</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>(16,18)</t>
+          <t>(7,9)</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2272,7 +2272,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2281,21 +2281,21 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.004141846612062547</v>
+        <v>0.006896551724137931</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>BALBc|SNY</t>
+          <t>BALBc|RTY</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>(17,18)</t>
+          <t>(8,9)</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2314,30 +2314,30 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>0.00558477823235275</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>B10BRF|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>(19,20)</t>
+          <t>(10,11)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2356,30 +2356,30 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>0.01888810884899542</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>B10BRF|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>(19,21)</t>
+          <t>(10,12)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2398,30 +2398,30 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>B10BRF</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.0005387931034482759</v>
+        <v>0.009592102812441796</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>B10BRF|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>(20,21)</t>
+          <t>(10,13)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2440,30 +2440,30 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.00202020202020202</v>
+        <v>0.0005579967915184488</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>B10BRM|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>(22,23)</t>
+          <t>(10,14)</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2482,30 +2482,30 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.0007471980074719801</v>
+        <v>0.004266113224950997</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>B10BRM|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>(22,24)</t>
+          <t>(10,15)</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2524,30 +2524,30 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>B10BRM</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.0006408715853560842</v>
+        <v>0.008229613004148813</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>B10BRM|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>(23,24)</t>
+          <t>(11,12)</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2566,30 +2566,30 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.0004705882352941177</v>
+        <v>0.005368195023367437</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>BALBc|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>(25,26)</t>
+          <t>(11,13)</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2608,30 +2608,30 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>0.02969348659003831</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>BALBc|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>(25,27)</t>
+          <t>(11,14)</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2650,30 +2650,30 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.005313092979127135</v>
+        <v>0.005786222534991008</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>BALBc|VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>(26,27)</t>
+          <t>(11,15)</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2685,45 +2685,41 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>0.01219195006177255</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>B10BR|RTY × BALBc|RTY</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>BALBc</t>
-        </is>
-      </c>
+          <t>(12,13)</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
@@ -2731,8 +2727,8 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2741,13 +2737,17 @@
           <t>SNY</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>0.009277522098034919</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2757,19 +2757,11 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>B10BR|SNY × BALBc|SNY</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>BALBc</t>
-        </is>
-      </c>
+          <t>(12,14)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
@@ -2777,45 +2769,41 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>VGP</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
       <c r="E58" t="n">
-        <v>0.0005690102777481419</v>
+        <v>0.005434126313247192</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>VGP</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>B10BR|VGP × BALBc|VGP</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>BALBc</t>
-        </is>
-      </c>
+          <t>(12,15)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
@@ -2823,316 +2811,293 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>B10BR</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.001212469289429182</v>
+        <v>0.001865418532085199</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>B10BR|RTY × B10BR|SNY</t>
+          <t>(13,14)</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>SNY</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
           <t>B10BR</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.0001587793926503604</v>
+        <v>0.005793526201689467</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>B10BR|RTY × B10BR|VGP</t>
+          <t>(13,15)</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>VGP</t>
-        </is>
-      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>B10BR</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.0001263573222030195</v>
+        <v>0.001847652641303435</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>B10BR|SNY</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>B10BR</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>B10BR|SNY × B10BR|VGP</t>
+          <t>(14,15)</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>SNY</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>VGP</t>
-        </is>
-      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>BALBc</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.004293738298314957</v>
+        <v>0.005734666759913281</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>BALBc|SNY</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>BALBc|RTY × BALBc|SNY</t>
+          <t>(16,17)</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>SNY</t>
-        </is>
-      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>BALBc</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.002328050449620732</v>
+        <v>0.005484237894052649</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>BALBc|SNY</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>BALBc|RTY × BALBc|VGP</t>
+          <t>(16,18)</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>VGP</t>
-        </is>
-      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
           <t>BALBc</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.004387668199625277</v>
+        <v>0.004141846612062547</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>BALBc|SNY</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>BALBc|SNY × BALBc|VGP</t>
+          <t>(17,18)</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>SNY</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>VGP</t>
-        </is>
-      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>L5: all supersets</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
       <c r="E65" t="n">
-        <v>3.996166178072911e-05</v>
+        <v>0</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>B10BR × BALBc</t>
+          <t>B10BR|VGP</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>B10BR × BALBc</t>
+          <t>VGP</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>B10BR × BALBc</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>BALBc</t>
-        </is>
-      </c>
+          <t>(19,20)</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
@@ -3140,154 +3105,1323 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>L6: pre-immune</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr">
         <is>
           <t>B10BR</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>2.421027674426409e-08</v>
+        <v>0</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>B10BR SLO</t>
+          <t>B10BR|VGP</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>B10BR SLO</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr"/>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>(19,21)</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>individual</t>
-        </is>
-      </c>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>L6: pre-immune</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1.949841837061067e-08</v>
+        <v>0.02492163009404389</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>BALBc SLO</t>
+          <t>B10BR|VGP</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>BALBc SLO</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>(19,22)</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>individual</t>
-        </is>
-      </c>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>L6: pre-immune</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>B10BR × BALBc</t>
+          <t>B10BR</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>8.7710385535849e-10</v>
+        <v>0</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>B10BR × BALBc SLO</t>
+          <t>B10BR|VGP</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>B10BR × BALBc SLO</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr"/>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>(19,23)</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>cross</t>
-        </is>
-      </c>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>L5: all supersets</t>
+          <t>L2: within superset
+across mice</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
       <c r="E69" t="n">
         <v>0</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>B10BR Kb × B10BR Kd</t>
+          <t>B10BR|VGP</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>B10BR Kb × B10BR Kd</t>
+          <t>VGP</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>B10BR Kb × B10BR Kd</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>B10BR</t>
-        </is>
-      </c>
+          <t>(19,24)</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.0005387931034482759</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>(20,21)</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0.001763322884012539</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>(20,22)</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0.0002520669489816495</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>(20,23)</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0.01794992914501653</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>(20,24)</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>0.0004261363636363636</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>(21,22)</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>(21,23)</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>0.0004280821917808219</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>(21,24)</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>0.00202020202020202</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>(22,23)</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>0.0007471980074719801</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>(22,24)</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>0.0006408715853560842</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>(23,24)</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>0.0004705882352941177</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>(25,26)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>(25,27)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>L2: within superset
+across mice</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>0.005313092979127135</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>(26,27)</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>L3: within epitope
+across strain</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>B10BR|RTY × BALBc|RTY</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>L3: within epitope
+across strain</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>B10BR|SNY × BALBc|SNY</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>L3: within epitope
+across strain</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>0.0005690102777481419</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>B10BR|VGP × BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>0.001212469289429182</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>B10BR|RTY × B10BR|SNY</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>0.0001587793926503604</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>B10BR|RTY × B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0.0001263573222030195</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>B10BR|SNY × B10BR|VGP</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>0.004293738298314957</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>BALBc|RTY × BALBc|SNY</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>0.002328050449620732</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>BALBc|RTY × BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>L4: within strain
+across epitope</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0.004387668199625277</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>BALBc|SNY × BALBc|VGP</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>VGP</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>L5: all supersets</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>3.996166178072911e-05</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>L6: pre-immune</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2.421027674426409e-08</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>B10BR SLO</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>B10BR SLO</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>L6: pre-immune</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>BALBc</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1.949841837061067e-08</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>BALBc SLO</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>BALBc SLO</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>L6: pre-immune</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>8.7710385535849e-10</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc SLO</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>B10BR × BALBc SLO</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>cross</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>L5: all supersets</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>B10BR Kb × B10BR Kd</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>B10BR Kb × B10BR Kd</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>B10BR Kb × B10BR Kd</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>B10BR</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
this is what i just updated lol
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Superset/Kb_pc_values_CDR3.xlsx
+++ b/Final_Figures_and_Sheets_Superset/Kb_pc_values_CDR3.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -537,7 +537,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -576,7 +576,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -615,7 +615,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -654,7 +654,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -693,7 +693,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -732,7 +732,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -771,7 +771,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -810,7 +810,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -849,7 +849,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -888,7 +888,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -927,7 +927,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -966,7 +966,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1005,7 +1005,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1044,7 +1044,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1083,7 +1083,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1122,7 +1122,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1161,7 +1161,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1200,7 +1200,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1239,7 +1239,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1278,7 +1278,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1317,7 +1317,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1356,7 +1356,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1395,7 +1395,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1434,7 +1434,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1473,7 +1473,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1512,7 +1512,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>L1: within sample</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1551,8 +1551,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1593,8 +1592,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1635,8 +1633,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1677,8 +1674,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1719,8 +1715,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1761,8 +1756,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1803,8 +1797,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1845,8 +1838,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1887,8 +1879,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1929,8 +1920,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1971,8 +1961,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -2013,8 +2002,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -2055,8 +2043,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -2097,8 +2084,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -2139,8 +2125,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2181,8 +2166,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2223,8 +2207,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -2265,8 +2248,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -2307,8 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -2349,8 +2330,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -2391,8 +2371,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2433,8 +2412,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2475,8 +2453,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2517,8 +2494,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2559,8 +2535,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -2601,8 +2576,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -2643,8 +2617,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -2685,8 +2658,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -2727,8 +2699,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2769,8 +2740,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -2811,8 +2781,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -2853,8 +2822,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -2895,8 +2863,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -2937,8 +2904,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -2979,8 +2945,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -3021,8 +2986,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -3063,8 +3027,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -3105,8 +3068,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -3147,8 +3109,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -3189,8 +3150,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -3231,8 +3191,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
@@ -3273,8 +3232,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -3315,8 +3273,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
@@ -3357,8 +3314,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
@@ -3399,8 +3355,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
@@ -3441,8 +3396,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
@@ -3483,8 +3437,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
@@ -3525,8 +3478,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
@@ -3567,8 +3519,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -3609,8 +3560,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -3651,8 +3601,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
@@ -3693,8 +3642,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
@@ -3735,8 +3683,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
@@ -3777,8 +3724,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>L2: within superset
-across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
@@ -3819,8 +3765,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
@@ -3865,8 +3810,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -3911,8 +3855,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>L3: within epitope
-across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -3957,8 +3900,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -4003,8 +3945,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -4049,8 +3990,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -4095,8 +4035,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -4141,8 +4080,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -4187,8 +4125,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>L4: within strain
-across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -4233,7 +4170,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>L5: all supersets</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -4348,7 +4285,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>L6: pre-immune</t>
+          <t>Pre-immune repertoires</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -4385,7 +4322,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>L5: all supersets</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>

</xml_diff>